<commit_message>
Expand Blue Goat best-fit picks with live Semrush verification
Full best-fit list (39 sites) across medical/health-IT/medtech/science and
tech/cybersecurity/software/engineering, not already built. Top 12 verified
with live Semrush Authority Score (sheet metrics confirmed accurate within
1-2 pts). Includes AS/TF/Traffic/RD/Price and fit notes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EyZhZSnP6QyNR5y5EJdqhU
</commit_message>
<xml_diff>
--- a/bluegoatcyber-selected-links.xlsx
+++ b/bluegoatcyber-selected-links.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="BlueGoat tech-health picks" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BlueGoat best-fit picks" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,17 +423,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,672 +450,1348 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>AS</t>
+          <t>AS (sheet)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>AS (live Semrush)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>TF</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Traffic</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Price ($)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Ref Domains</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Verdict</t>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Fit note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>biospace.com</t>
+          <t>medindia.net</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Medical/Life-Sci</t>
+          <t>Medical</t>
         </is>
       </c>
       <c r="C2" t="n">
+        <v>61</v>
+      </c>
+      <c r="D2" t="n">
+        <v>62</v>
+      </c>
+      <c r="E2" t="n">
         <v>49</v>
       </c>
-      <c r="D2" t="n">
-        <v>63</v>
-      </c>
-      <c r="E2" t="n">
-        <v>92436</v>
-      </c>
       <c r="F2" t="n">
-        <v>805</v>
+        <v>613038</v>
       </c>
       <c r="G2" t="n">
-        <v>29719</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>BUY - biotech/pharma/clinical, ideal audience</t>
+        <v>250</v>
+      </c>
+      <c r="H2" t="n">
+        <v>19125</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>medical info, cheap</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>medindia.net</t>
+          <t>zmescience.com</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Medical/Health</t>
+          <t>Science</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>61</v>
-      </c>
-      <c r="D3" t="n">
-        <v>49</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="n">
-        <v>613038</v>
+        <v>52</v>
       </c>
       <c r="F3" t="n">
-        <v>250</v>
+        <v>101131</v>
       </c>
       <c r="G3" t="n">
-        <v>19125</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>BUY - medical, cheap</t>
+        <v>620</v>
+      </c>
+      <c r="H3" t="n">
+        <v>25026</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>science/tech</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>beckershospitalreview.com</t>
+          <t>biospace.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Medical/Health</t>
+          <t>Life-Sci</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D4" t="n">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E4" t="n">
-        <v>64994</v>
+        <v>63</v>
       </c>
       <c r="F4" t="n">
-        <v>4560</v>
+        <v>92436</v>
       </c>
       <c r="G4" t="n">
-        <v>34867</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>BUY (premium) - top healthcare trade</t>
+        <v>805</v>
+      </c>
+      <c r="H4" t="n">
+        <v>29719</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>★ biotech/pharma/clinical audience</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>zmescience.com</t>
+          <t>microbenotes.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Science</t>
+          <t>Science/Med</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51</v>
-      </c>
-      <c r="D5" t="n">
-        <v>52</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>101131</v>
+        <v>24</v>
       </c>
       <c r="F5" t="n">
-        <v>620</v>
+        <v>796212</v>
       </c>
       <c r="G5" t="n">
-        <v>25026</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>BUY - science/tech</t>
+        <v>350</v>
+      </c>
+      <c r="H5" t="n">
+        <v>7862</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>science/medicine/research</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>psypost.org</t>
+          <t>clinicspots.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Health-Science</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>48</v>
-      </c>
-      <c r="D6" t="n">
-        <v>35</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>22950</v>
+        <v>21</v>
       </c>
       <c r="F6" t="n">
-        <v>1330</v>
+        <v>133460</v>
       </c>
       <c r="G6" t="n">
-        <v>24379</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Consider - psychology/science</t>
+        <v>350</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4414</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>healthcare</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>homecaremag.com</t>
+          <t>drlogy.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Medical/Business</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>32</v>
-      </c>
-      <c r="D7" t="n">
-        <v>48</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
-        <v>3881</v>
+        <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>3145</v>
+        <v>439834</v>
       </c>
       <c r="G7" t="n">
-        <v>2562</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Consider - health/medical business</t>
+        <v>470</v>
+      </c>
+      <c r="H7" t="n">
+        <v>7181</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>healthcare/medical info</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>zdnet.com</t>
+          <t>blog.medicai.io</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tech/Enterprise</t>
+          <t>Medical-Imaging</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="D8" t="n">
-        <v>84</v>
+        <v>43</v>
       </c>
       <c r="E8" t="n">
-        <v>976673</v>
+        <v>15</v>
       </c>
       <c r="F8" t="n">
-        <v>3613</v>
+        <v>60685</v>
       </c>
       <c r="G8" t="n">
-        <v>215869</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>BUY - enterprise tech/security news</t>
+        <v>520</v>
+      </c>
+      <c r="H8" t="n">
+        <v>310</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>★ imaging/telemedicine (DICOM angle)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cnet.com</t>
+          <t>media.market.us</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Tech/Media</t>
+          <t>News/Tech/Health</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>85</v>
-      </c>
-      <c r="D9" t="n">
-        <v>86</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>12969237</v>
+        <v>25</v>
       </c>
       <c r="F9" t="n">
-        <v>3841</v>
+        <v>23323</v>
       </c>
       <c r="G9" t="n">
-        <v>493456</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>BUY (premium) - major tech media</t>
+        <v>450</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3010</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>tech+health+business news</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sourceforge.net</t>
+          <t>eletsonline.com</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tech/Software</t>
+          <t>Health/Gov</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>76</v>
-      </c>
-      <c r="D10" t="n">
-        <v>95</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="n">
-        <v>5361290</v>
+        <v>32</v>
       </c>
       <c r="F10" t="n">
-        <v>3375</v>
+        <v>78769</v>
       </c>
       <c r="G10" t="n">
-        <v>273832</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>BUY - software authority</t>
+        <v>542</v>
+      </c>
+      <c r="H10" t="n">
+        <v>6744</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>health/e-gov</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dev.to</t>
+          <t>radiologykey.com</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tech/Dev</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="D11" t="n">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="E11" t="n">
-        <v>2011489</v>
+        <v>23</v>
       </c>
       <c r="F11" t="n">
-        <v>70</v>
+        <v>147633</v>
       </c>
       <c r="G11" t="n">
-        <v>123886</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>BUY - dev audience, great value</t>
+        <v>250</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4004</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>radiology/imaging reference</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>acm.org</t>
+          <t>medcitynews.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Tech/Computing</t>
+          <t>Health-Tech</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D12" t="n">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="E12" t="n">
-        <v>761786</v>
+        <v>32</v>
       </c>
       <c r="F12" t="n">
-        <v>1144</v>
+        <v>10298</v>
       </c>
       <c r="G12" t="n">
-        <v>177659</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>BUY - computing body, high trust</t>
+        <v>5210</v>
+      </c>
+      <c r="H12" t="n">
+        <v>17849</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>★ health/tech/news</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>slashdot.org</t>
+          <t>medicaldaily.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tech/Security</t>
+          <t>Health-Science</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>56</v>
-      </c>
-      <c r="D13" t="n">
-        <v>71</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>198658</v>
+        <v>35</v>
       </c>
       <c r="F13" t="n">
-        <v>2640</v>
+        <v>8205</v>
       </c>
       <c r="G13" t="n">
-        <v>124410</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>BUY - tech/security/software news</t>
+        <v>1320</v>
+      </c>
+      <c r="H13" t="n">
+        <v>34888</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>health/science news</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sitepoint.com</t>
+          <t>electroiq.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tech/Dev</t>
+          <t>Electronics</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>54</v>
-      </c>
-      <c r="D14" t="n">
-        <v>74</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="n">
-        <v>249489</v>
+        <v>28</v>
       </c>
       <c r="F14" t="n">
-        <v>1650</v>
+        <v>5411</v>
       </c>
       <c r="G14" t="n">
-        <v>44357</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>BUY - web/software dev</t>
+        <v>380</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7740</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>semiconductors/devices + health</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>techtimes.com</t>
+          <t>healthcare-digital.com</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Health-IT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="D15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E15" t="n">
-        <v>75454</v>
+        <v>26</v>
       </c>
       <c r="F15" t="n">
-        <v>975</v>
+        <v>12644</v>
       </c>
       <c r="G15" t="n">
-        <v>46764</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>BUY - tech news, value</t>
+        <v>5215</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2787</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>★ healthcare + technology</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>freecodecamp.org</t>
+          <t>pharmaphorum.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tech/Education</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="D16" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E16" t="n">
-        <v>2428426</v>
+        <v>32</v>
       </c>
       <c r="F16" t="n">
-        <v>775</v>
+        <v>7931</v>
       </c>
       <c r="G16" t="n">
-        <v>70630</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>BUY - programming/education</t>
+        <v>583</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8343</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>pharma industry</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>filehippo.com</t>
+          <t>pharmatimes.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tech/Software</t>
+          <t>Pharma</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>65</v>
-      </c>
-      <c r="D17" t="n">
-        <v>67</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2411631</v>
+        <v>27</v>
       </c>
       <c r="F17" t="n">
-        <v>3120</v>
+        <v>11320</v>
       </c>
       <c r="G17" t="n">
-        <v>48236</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Consider - software</t>
+        <v>2868</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5562</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>pharma news</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>appleinsider.com</t>
+          <t>healthcareittoday.com</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tech</t>
+          <t>Health-IT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="D18" t="n">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="E18" t="n">
-        <v>467492</v>
+        <v>29</v>
       </c>
       <c r="F18" t="n">
-        <v>21250</v>
+        <v>15243</v>
       </c>
       <c r="G18" t="n">
-        <v>73162</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Skip - $21k, low relevance</t>
+        <v>1960</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4187</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>★ ideal - healthcare IT news</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bizjournals.com</t>
+          <t>clinicalgate.com</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Business</t>
+          <t>Medical-Ref</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>56</v>
-      </c>
-      <c r="D19" t="n">
-        <v>70</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="n">
-        <v>1032102</v>
+        <v>23</v>
       </c>
       <c r="F19" t="n">
-        <v>2843</v>
+        <v>10428</v>
       </c>
       <c r="G19" t="n">
-        <v>214810</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Consider - US business (DR filler)</t>
+        <v>175</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2729</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>clinical/medical reference</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>thehindubusinessline.com</t>
+          <t>homehealthcarenews.com</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Business/Tech</t>
+          <t>Health-Biz</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>72</v>
-      </c>
-      <c r="D20" t="n">
-        <v>62</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>3251880</v>
+        <v>28</v>
       </c>
       <c r="F20" t="n">
-        <v>3910</v>
+        <v>4658</v>
       </c>
       <c r="G20" t="n">
-        <v>49949</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Consider - business/tech (India)</t>
+        <v>3900</v>
+      </c>
+      <c r="H20" t="n">
+        <v>4551</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>home health business</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>taipeitimes.com</t>
+          <t>sourceforge.net</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Business/AI</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="C21" t="n">
+        <v>76</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>95</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5361290</v>
+      </c>
+      <c r="G21" t="n">
+        <v>3375</v>
+      </c>
+      <c r="H21" t="n">
+        <v>273832</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>software authority</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>freecodecamp.org</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Programming</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>71</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>44</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2428426</v>
+      </c>
+      <c r="G22" t="n">
+        <v>775</v>
+      </c>
+      <c r="H22" t="n">
+        <v>70630</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>programming/education</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>dev.to</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>68</v>
+      </c>
+      <c r="D23" t="n">
+        <v>69</v>
+      </c>
+      <c r="E23" t="n">
+        <v>55</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2011489</v>
+      </c>
+      <c r="G23" t="n">
+        <v>70</v>
+      </c>
+      <c r="H23" t="n">
+        <v>123886</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>★ developer community, great value</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>tutorialspoint.com</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Programming</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>68</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>37</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1664817</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2875</v>
+      </c>
+      <c r="H24" t="n">
+        <v>51158</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>programming/education</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cybernews.com</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>65</v>
+      </c>
+      <c r="D25" t="n">
+        <v>62</v>
+      </c>
+      <c r="E25" t="n">
+        <v>35</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3416624</v>
+      </c>
+      <c r="G25" t="n">
+        <v>582</v>
+      </c>
+      <c r="H25" t="n">
+        <v>39175</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>★★ dedicated cybersecurity</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>filehippo.com</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>65</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>67</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2411631</v>
+      </c>
+      <c r="G26" t="n">
+        <v>3120</v>
+      </c>
+      <c r="H26" t="n">
+        <v>48236</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>software</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>clickup.com</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SaaS/Tech</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>65</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>40</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1789240</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2350</v>
+      </c>
+      <c r="H27" t="n">
+        <v>78557</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>productivity/tech (UGC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>acm.org</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Computing</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>60</v>
+      </c>
+      <c r="D28" t="n">
+        <v>60</v>
+      </c>
+      <c r="E28" t="n">
+        <v>83</v>
+      </c>
+      <c r="F28" t="n">
+        <v>761786</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1144</v>
+      </c>
+      <c r="H28" t="n">
+        <v>177659</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>★ computing body, high trust</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>slashdot.org</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tech/Security</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>56</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>71</v>
+      </c>
+      <c r="F29" t="n">
+        <v>198658</v>
+      </c>
+      <c r="G29" t="n">
+        <v>2640</v>
+      </c>
+      <c r="H29" t="n">
+        <v>124410</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>tech/security/software news</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sitepoint.com</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
         <v>54</v>
       </c>
-      <c r="D21" t="n">
-        <v>66</v>
-      </c>
-      <c r="E21" t="n">
-        <v>146080</v>
-      </c>
-      <c r="F21" t="n">
-        <v>3496</v>
-      </c>
-      <c r="G21" t="n">
-        <v>37543</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Consider - business/AI</t>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>74</v>
+      </c>
+      <c r="F30" t="n">
+        <v>249489</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1650</v>
+      </c>
+      <c r="H30" t="n">
+        <v>44357</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>web/software dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>thebestvpn.com</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>52</v>
+      </c>
+      <c r="D31" t="n">
+        <v>55</v>
+      </c>
+      <c r="E31" t="n">
+        <v>43</v>
+      </c>
+      <c r="F31" t="n">
+        <v>418412</v>
+      </c>
+      <c r="G31" t="n">
+        <v>4300</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3664</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>★ security/VPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>techtimes.com</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>50</v>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>35</v>
+      </c>
+      <c r="F32" t="n">
+        <v>75454</v>
+      </c>
+      <c r="G32" t="n">
+        <v>975</v>
+      </c>
+      <c r="H32" t="n">
+        <v>46764</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>tech news, value</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>digitimes.com</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Tech/Hardware</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>45</v>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>53</v>
+      </c>
+      <c r="F33" t="n">
+        <v>19373</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1250</v>
+      </c>
+      <c r="H33" t="n">
+        <v>25042</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>tech/hardware/supply chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>c-sharpcorner.com</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Programming</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>43</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>60</v>
+      </c>
+      <c r="F34" t="n">
+        <v>98016</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1340</v>
+      </c>
+      <c r="H34" t="n">
+        <v>20686</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>programming/dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>automation.com</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Automation</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>41</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>55</v>
+      </c>
+      <c r="F35" t="n">
+        <v>17851</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1715</v>
+      </c>
+      <c r="H35" t="n">
+        <v>9856</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>★ industrial automation/embedded</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>afcea.org</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Defense/Security</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>41</v>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>55</v>
+      </c>
+      <c r="F36" t="n">
+        <v>14826</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2355</v>
+      </c>
+      <c r="H36" t="n">
+        <v>7942</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>★ defense/security comms assoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>designnews.com</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>41</v>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>55</v>
+      </c>
+      <c r="F37" t="n">
+        <v>16139</v>
+      </c>
+      <c r="G37" t="n">
+        <v>9750</v>
+      </c>
+      <c r="H37" t="n">
+        <v>10635</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>device/engineering (premium $)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>cyberpanel.net</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Security/Hosting</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>40</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>67</v>
+      </c>
+      <c r="F38" t="n">
+        <v>30721</v>
+      </c>
+      <c r="G38" t="n">
+        <v>450</v>
+      </c>
+      <c r="H38" t="n">
+        <v>35935</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>web security/hosting</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>thewindowsclub.com</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>40</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>57</v>
+      </c>
+      <c r="F39" t="n">
+        <v>10870</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2125</v>
+      </c>
+      <c r="H39" t="n">
+        <v>25996</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Windows/tech</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>osnews.com</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Tech/OS</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>39</v>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>63</v>
+      </c>
+      <c r="F40" t="n">
+        <v>12102</v>
+      </c>
+      <c r="G40" t="n">
+        <v>760</v>
+      </c>
+      <c r="H40" t="n">
+        <v>12508</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>tech/software/OS news</t>
         </is>
       </c>
     </row>

</xml_diff>